<commit_message>
Update 2026-07-15 - added  tags to RFP requests and added that tag to the auto-exclude criteria
</commit_message>
<xml_diff>
--- a/scorecard.xlsx
+++ b/scorecard.xlsx
@@ -967,18 +967,18 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-30 05:00</t>
+          <t>2026-07-15 05:00</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -1643,12 +1643,12 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -3520,18 +3520,18 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-06-30 05:00</t>
+          <t>2026-07-15 05:00</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -5092,12 +5092,12 @@
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
@@ -5425,12 +5425,12 @@
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>120</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
@@ -6085,12 +6085,12 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>132</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr">
@@ -7528,12 +7528,12 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S71" s="3" t="inlineStr">
@@ -8351,7 +8351,7 @@
         <v/>
       </c>
       <c r="Y71" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z71" s="3" t="n"/>
     </row>
@@ -8435,7 +8435,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S72" s="3" t="inlineStr">
@@ -8462,7 +8462,7 @@
         <v/>
       </c>
       <c r="Y72" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z72" s="3" t="n"/>
     </row>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S73" s="3" t="inlineStr">
@@ -8573,7 +8573,7 @@
         <v/>
       </c>
       <c r="Y73" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z73" s="3" t="n"/>
     </row>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S74" s="3" t="inlineStr">
@@ -8684,7 +8684,7 @@
         <v/>
       </c>
       <c r="Y74" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z74" s="3" t="n"/>
     </row>
@@ -8753,12 +8753,12 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q75" s="2" t="inlineStr">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S75" s="3" t="inlineStr">
@@ -8795,7 +8795,7 @@
         <v/>
       </c>
       <c r="Y75" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z75" s="3" t="n"/>
     </row>
@@ -8868,12 +8868,12 @@
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q76" s="2" t="inlineStr">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S76" s="3" t="inlineStr">
@@ -8910,7 +8910,7 @@
         <v/>
       </c>
       <c r="Y76" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z76" s="3" t="n"/>
     </row>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-citizen</t>
+          <t>transparent-nh, nh-citizen, nh-rfp</t>
         </is>
       </c>
       <c r="S77" s="3" t="inlineStr">
@@ -9019,7 +9019,7 @@
         <v/>
       </c>
       <c r="Y77" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z77" s="3" t="n"/>
     </row>
@@ -9103,7 +9103,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-citizen</t>
+          <t>transparent-nh, nh-citizen, nh-rfp</t>
         </is>
       </c>
       <c r="S78" s="3" t="inlineStr">
@@ -9130,7 +9130,7 @@
         <v/>
       </c>
       <c r="Y78" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z78" s="3" t="n"/>
     </row>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S79" s="3" t="inlineStr">
@@ -9241,7 +9241,7 @@
         <v/>
       </c>
       <c r="Y79" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z79" s="3" t="n"/>
     </row>
@@ -9310,12 +9310,12 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="Q80" s="2" t="inlineStr">
@@ -9325,7 +9325,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S80" s="3" t="inlineStr">
@@ -9434,7 +9434,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S81" s="3" t="inlineStr">
@@ -9461,7 +9461,7 @@
         <v/>
       </c>
       <c r="Y81" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z81" s="3" t="n"/>
     </row>
@@ -9545,7 +9545,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-citizen</t>
+          <t>transparent-nh, nh-citizen, nh-rfp</t>
         </is>
       </c>
       <c r="S82" s="3" t="inlineStr">
@@ -9572,7 +9572,7 @@
         <v/>
       </c>
       <c r="Y82" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z82" s="3" t="n"/>
     </row>
@@ -9656,7 +9656,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S83" s="3" t="inlineStr">
@@ -9681,7 +9681,7 @@
         <v/>
       </c>
       <c r="Y83" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z83" s="3" t="n"/>
     </row>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson, nh-pickedup</t>
+          <t>transparent-nh, nh-inperson, nh-pickedup, nh-rfp</t>
         </is>
       </c>
       <c r="S84" s="3" t="inlineStr">
@@ -9792,7 +9792,7 @@
         <v/>
       </c>
       <c r="Y84" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z84" s="3" t="n"/>
     </row>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S85" s="3" t="inlineStr">
@@ -9901,7 +9901,7 @@
         <v/>
       </c>
       <c r="Y85" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z85" s="3" t="n"/>
     </row>
@@ -9974,12 +9974,12 @@
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="Q86" s="2" t="inlineStr">
@@ -9989,7 +9989,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S86" s="3" t="inlineStr">
@@ -10083,12 +10083,12 @@
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>137</t>
         </is>
       </c>
       <c r="Q87" s="2" t="inlineStr">
@@ -10098,7 +10098,7 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S87" s="3" t="inlineStr">
@@ -10123,7 +10123,7 @@
         <v/>
       </c>
       <c r="Y87" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z87" s="3" t="n"/>
     </row>
@@ -10207,7 +10207,7 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S88" s="3" t="inlineStr">
@@ -10234,7 +10234,7 @@
         <v/>
       </c>
       <c r="Y88" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z88" s="3" t="n"/>
     </row>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-citizen, nh-inperson</t>
+          <t>transparent-nh, nh-citizen, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S89" s="3" t="inlineStr">
@@ -10345,7 +10345,7 @@
         <v/>
       </c>
       <c r="Y89" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z89" s="3" t="n"/>
     </row>
@@ -10429,7 +10429,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-citizen</t>
+          <t>transparent-nh, nh-citizen, nh-rfp</t>
         </is>
       </c>
       <c r="S90" s="3" t="inlineStr">
@@ -10456,7 +10456,7 @@
         <v/>
       </c>
       <c r="Y90" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z90" s="3" t="n"/>
     </row>
@@ -10525,12 +10525,12 @@
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>120</t>
         </is>
       </c>
       <c r="Q91" s="2" t="inlineStr">
@@ -10540,7 +10540,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S91" s="3" t="inlineStr">
@@ -10565,7 +10565,7 @@
         <v/>
       </c>
       <c r="Y91" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z91" s="3" t="n"/>
     </row>
@@ -10634,12 +10634,12 @@
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="Q92" s="2" t="inlineStr">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>transparent-nh</t>
+          <t>transparent-nh, nh-rfp</t>
         </is>
       </c>
       <c r="S92" s="3" t="inlineStr">
@@ -10676,7 +10676,7 @@
         <v/>
       </c>
       <c r="Y92" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z92" s="3" t="n"/>
     </row>
@@ -10758,7 +10758,11 @@
           <t>https://www.muckrock.com/foi/troy-4012/highest-value-rfps-troy-clerk-200680/</t>
         </is>
       </c>
-      <c r="R93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>nh-rfp</t>
+        </is>
+      </c>
       <c r="S93" s="3" t="inlineStr">
         <is>
           <t>Troy</t>
@@ -10783,7 +10787,7 @@
         <v/>
       </c>
       <c r="Y93" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z93" s="3" t="n"/>
     </row>
@@ -10963,12 +10967,12 @@
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q95" s="2" t="inlineStr">
@@ -11074,12 +11078,12 @@
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="Q96" s="2" t="inlineStr">
@@ -11294,12 +11298,12 @@
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="Q98" s="2" t="inlineStr">
@@ -11623,12 +11627,12 @@
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q101" s="2" t="inlineStr">
@@ -12178,12 +12182,12 @@
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="Q106" s="2" t="inlineStr">
@@ -12289,12 +12293,12 @@
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="Q107" s="2" t="inlineStr">
@@ -12400,12 +12404,12 @@
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>70</t>
         </is>
       </c>
       <c r="Q108" s="2" t="inlineStr">
@@ -12842,12 +12846,12 @@
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q112" s="2" t="inlineStr">
@@ -13288,12 +13292,12 @@
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q116" s="2" t="inlineStr">
@@ -13843,12 +13847,12 @@
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q121" s="2" t="inlineStr">
@@ -14404,12 +14408,12 @@
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -14513,12 +14517,12 @@
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q127" s="2" t="inlineStr">
@@ -14622,12 +14626,12 @@
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
@@ -15173,12 +15177,12 @@
       <c r="N133" t="inlineStr"/>
       <c r="O133" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q133" s="2" t="inlineStr">
@@ -15284,12 +15288,12 @@
       <c r="N134" t="inlineStr"/>
       <c r="O134" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -15395,12 +15399,12 @@
       <c r="N135" t="inlineStr"/>
       <c r="O135" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="Q135" s="2" t="inlineStr">
@@ -15617,12 +15621,12 @@
       <c r="N137" t="inlineStr"/>
       <c r="O137" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="Q137" s="2" t="inlineStr">
@@ -15835,12 +15839,12 @@
       <c r="N139" t="inlineStr"/>
       <c r="O139" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="Q139" s="2" t="inlineStr">
@@ -17837,12 +17841,12 @@
       <c r="N157" t="inlineStr"/>
       <c r="O157" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>114</t>
         </is>
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="Q157" s="2" t="inlineStr">
@@ -19284,12 +19288,12 @@
       <c r="N170" t="inlineStr"/>
       <c r="O170" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>116</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
       <c r="Q170" s="2" t="inlineStr">
@@ -20402,12 +20406,12 @@
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>116</t>
         </is>
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
       <c r="Q180" s="2" t="inlineStr">
@@ -21516,12 +21520,12 @@
       <c r="N190" t="inlineStr"/>
       <c r="O190" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr">
@@ -21738,12 +21742,12 @@
       <c r="N192" t="inlineStr"/>
       <c r="O192" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="Q192" s="2" t="inlineStr">
@@ -21847,12 +21851,12 @@
       <c r="N193" t="inlineStr"/>
       <c r="O193" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="Q193" s="2" t="inlineStr">
@@ -23294,12 +23298,12 @@
       <c r="N206" t="inlineStr"/>
       <c r="O206" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Q206" s="2" t="inlineStr">
@@ -24400,12 +24404,12 @@
       <c r="N216" t="inlineStr"/>
       <c r="O216" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>131</t>
         </is>
       </c>
       <c r="P216" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="Q216" s="2" t="inlineStr">
@@ -24620,12 +24624,12 @@
       <c r="N218" t="inlineStr"/>
       <c r="O218" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>131</t>
         </is>
       </c>
       <c r="P218" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="Q218" s="2" t="inlineStr">
@@ -26180,12 +26184,12 @@
       <c r="N232" t="inlineStr"/>
       <c r="O232" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>131</t>
         </is>
       </c>
       <c r="P232" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>58</t>
         </is>
       </c>
       <c r="Q232" s="2" t="inlineStr">
@@ -26289,12 +26293,12 @@
       <c r="N233" t="inlineStr"/>
       <c r="O233" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q233" s="2" t="inlineStr">
@@ -26959,12 +26963,12 @@
       <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>80</t>
         </is>
       </c>
       <c r="Q239" s="2" t="inlineStr">
@@ -27288,12 +27292,12 @@
       <c r="N242" t="inlineStr"/>
       <c r="O242" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q242" s="2" t="inlineStr">
@@ -27847,12 +27851,12 @@
       <c r="N247" t="inlineStr"/>
       <c r="O247" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="Q247" s="2" t="inlineStr">
@@ -28957,12 +28961,12 @@
       <c r="N257" t="inlineStr"/>
       <c r="O257" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q257" s="2" t="inlineStr">
@@ -30075,12 +30079,12 @@
       <c r="N267" t="inlineStr"/>
       <c r="O267" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="Q267" s="2" t="inlineStr">
@@ -30739,12 +30743,12 @@
       <c r="N273" t="inlineStr"/>
       <c r="O273" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P273" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="Q273" s="2" t="inlineStr">
@@ -30850,12 +30854,12 @@
       <c r="N274" t="inlineStr"/>
       <c r="O274" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="Q274" s="2" t="inlineStr">
@@ -31294,12 +31298,12 @@
       <c r="N278" t="inlineStr"/>
       <c r="O278" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="Q278" s="2" t="inlineStr">
@@ -31640,7 +31644,7 @@
       </c>
       <c r="R281" t="inlineStr">
         <is>
-          <t>transparent-nh, nh-inperson</t>
+          <t>transparent-nh, nh-inperson, nh-rfp</t>
         </is>
       </c>
       <c r="S281" s="3" t="inlineStr">

</xml_diff>